<commit_message>
code to run the main experiment with bayesian calibration posterior
</commit_message>
<xml_diff>
--- a/data/scenarios.xlsx
+++ b/data/scenarios.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/plima/dev/genomic-surveillance-voi/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB1CACD-C21E-0348-8641-790887F3344C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2C3D92-9CCD-4A4A-8E1C-2320A09FDC2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19920" xr2:uid="{2F6A880A-CADF-8941-BACA-B4A1F43DB678}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19840" xr2:uid="{2F6A880A-CADF-8941-BACA-B4A1F43DB678}"/>
   </bookViews>
   <sheets>
-    <sheet name="one-way-scenarios" sheetId="4" r:id="rId1"/>
-    <sheet name="base-case" sheetId="1" r:id="rId2"/>
-    <sheet name="base-case-test" sheetId="3" r:id="rId3"/>
-    <sheet name="policy_profile" sheetId="5" r:id="rId4"/>
+    <sheet name="one-way-scenarios-uncertainty" sheetId="7" r:id="rId1"/>
+    <sheet name="one-way-scenarios" sheetId="4" r:id="rId2"/>
+    <sheet name="base-case" sheetId="1" r:id="rId3"/>
+    <sheet name="base-case-test" sheetId="3" r:id="rId4"/>
+    <sheet name="policy_profile" sheetId="5" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId5"/>
+    <externalReference r:id="rId6"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="48">
   <si>
     <t>Scenario</t>
   </si>
@@ -174,6 +175,18 @@
   </si>
   <si>
     <t>NPIs + 10-day ESS</t>
+  </si>
+  <si>
+    <t>c_mult</t>
+  </si>
+  <si>
+    <t>R0_mult</t>
+  </si>
+  <si>
+    <t>fixed_tau</t>
+  </si>
+  <si>
+    <t>tau_set</t>
   </si>
 </sst>
 </file>
@@ -651,6 +664,1021 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B5CB32D-7197-8B4D-8E5D-B08CDF00F964}">
+  <dimension ref="A1:O19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="5">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <f>[1]parameters!$D$30</f>
+        <v>13</v>
+      </c>
+      <c r="H2">
+        <f>[1]parameters!$D$24</f>
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <f>[1]parameters!$D$25</f>
+        <v>14</v>
+      </c>
+      <c r="J2">
+        <f>[1]parameters!$D$32</f>
+        <v>0.3</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2" s="4">
+        <f>[1]parameters!$D$6</f>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M2" s="2">
+        <f>[1]parameters!$D$10</f>
+        <v>0.25</v>
+      </c>
+      <c r="N2" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="6">
+        <f>10^5</f>
+        <v>100000</v>
+      </c>
+      <c r="G3">
+        <f>G$2</f>
+        <v>13</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:M19" si="0">H$2</f>
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L3" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M3" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N3" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="5">
+        <f>F$2</f>
+        <v>1</v>
+      </c>
+      <c r="G4" s="7">
+        <f>G$2-2</f>
+        <v>11</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L4" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M4" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N4" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="5">
+        <f>F$2</f>
+        <v>1</v>
+      </c>
+      <c r="G5" s="7">
+        <f>G$2-5</f>
+        <v>8</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L5" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M5" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N5" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="5">
+        <f>F$2</f>
+        <v>1</v>
+      </c>
+      <c r="G6" s="7">
+        <f>G$2-10</f>
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L6" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M6" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N6" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <f>D5+1</f>
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="5">
+        <f t="shared" ref="F7:F17" si="1">F$2</f>
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <f t="shared" ref="G7:G19" si="2">G$2-5</f>
+        <v>8</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L7" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M7" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N7" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <f>D7+1</f>
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8" s="7">
+        <f>K$2*0.5</f>
+        <v>0.5</v>
+      </c>
+      <c r="L8" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M8" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N8" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <f t="shared" ref="D9:D19" si="3">D8+1</f>
+        <v>4</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9" s="7">
+        <f>K$2*1.5</f>
+        <v>1.5</v>
+      </c>
+      <c r="L9" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M9" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N9" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="E10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L10" s="10">
+        <f>L$2*0.5</f>
+        <v>3.6649999999999999E-3</v>
+      </c>
+      <c r="M10" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N10" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L11" s="10">
+        <f>L$2*1.5</f>
+        <v>1.0995E-2</v>
+      </c>
+      <c r="M11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N11" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="E12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L12" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M12" s="9">
+        <f>M$2*1.5</f>
+        <v>0.375</v>
+      </c>
+      <c r="N12" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L13" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M13" s="9">
+        <f>M$2*0.5</f>
+        <v>0.125</v>
+      </c>
+      <c r="N13" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="E14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L14" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M14" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" s="8">
+        <f>0.9/5</f>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L15" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M15" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" s="8">
+        <f>0.5/5</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>30</v>
+      </c>
+      <c r="F16" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H16" s="7">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L16" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M16" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N16" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" s="5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H17" s="7">
+        <v>14</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L17" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M17" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N17" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="E18" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="6">
+        <f>F17*0.5</f>
+        <v>0.5</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H18">
+        <v>7</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L18" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M18" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N18" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" t="b">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="E19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="6">
+        <f>F17*1.5</f>
+        <v>1.5</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H19">
+        <v>7</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J19">
+        <v>1</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="L19" s="4">
+        <f t="shared" si="0"/>
+        <v>7.3299999999999997E-3</v>
+      </c>
+      <c r="M19" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="N19" t="b">
+        <f>FALSE</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13D08609-CB1A-DE4B-9664-56E1F1BD1B3E}">
   <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1658,7 +2686,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E5F186-D7CF-8746-A7C8-0082BF7A0D1C}">
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1795,7 +2823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7AB0DF1-70C7-124B-9A2F-8427C9818EE3}">
   <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1995,7 +3023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C032C89E-E4A5-B744-9378-57725A202560}">
   <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>